<commit_message>
rearranged data structure to match AEO
</commit_message>
<xml_diff>
--- a/input_files/population.xlsx
+++ b/input_files/population.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,25 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://utoronto-my.sharepoint.com/personal/ian_elder_mail_utoronto_ca/Documents/Documents/TEMOA/buildings_sector/input_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="8_{27172EC9-7910-4A78-8C20-C12BBCC49DB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{254DB462-CE6D-4330-B5AF-9B57A21665C0}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A1F4FCB6-EB9F-435E-A7B8-638927D142CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
-    <sheet name="ON" sheetId="3" r:id="rId1"/>
+    <sheet name="ON" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -36,17 +25,13 @@
     <t>year</t>
   </si>
   <si>
-    <t>population</t>
+    <t xml:space="preserve"> population </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
-  </numFmts>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -480,7 +465,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="43">
+  <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -523,14 +508,12 @@
     <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="42" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="42" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="43">
+  <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -558,7 +541,6 @@
     <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
     <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
     <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Comma" xfId="42" builtinId="3"/>
     <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
     <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
     <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
@@ -884,20 +866,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" customWidth="1"/>
-    <col min="2" max="2" width="15.28515625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="11" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
     </row>
@@ -905,7 +885,7 @@
       <c r="A2">
         <v>2000</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="1">
         <v>11683290</v>
       </c>
     </row>
@@ -913,7 +893,7 @@
       <c r="A3">
         <v>2001</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="1">
         <v>11897534</v>
       </c>
     </row>
@@ -921,7 +901,7 @@
       <c r="A4">
         <v>2002</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="1">
         <v>12094174</v>
       </c>
     </row>
@@ -929,7 +909,7 @@
       <c r="A5">
         <v>2003</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="1">
         <v>12245039</v>
       </c>
     </row>
@@ -937,7 +917,7 @@
       <c r="A6">
         <v>2004</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="1">
         <v>12391421</v>
       </c>
     </row>
@@ -945,7 +925,7 @@
       <c r="A7">
         <v>2005</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="1">
         <v>12528663</v>
       </c>
     </row>
@@ -953,7 +933,7 @@
       <c r="A8">
         <v>2006</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8" s="1">
         <v>12661878</v>
       </c>
     </row>
@@ -961,7 +941,7 @@
       <c r="A9">
         <v>2007</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" s="1">
         <v>12764806</v>
       </c>
     </row>
@@ -969,7 +949,7 @@
       <c r="A10">
         <v>2008</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="1">
         <v>12883583</v>
       </c>
     </row>
@@ -977,7 +957,7 @@
       <c r="A11">
         <v>2009</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="1">
         <v>12998345</v>
       </c>
     </row>
@@ -985,7 +965,7 @@
       <c r="A12">
         <v>2010</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12" s="1">
         <v>13135778</v>
       </c>
     </row>
@@ -993,7 +973,7 @@
       <c r="A13">
         <v>2011</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B13" s="1">
         <v>13261381</v>
       </c>
     </row>
@@ -1001,7 +981,7 @@
       <c r="A14">
         <v>2012</v>
       </c>
-      <c r="B14" s="2">
+      <c r="B14" s="1">
         <v>13390632</v>
       </c>
     </row>
@@ -1009,7 +989,7 @@
       <c r="A15">
         <v>2013</v>
       </c>
-      <c r="B15" s="2">
+      <c r="B15" s="1">
         <v>13510781</v>
       </c>
     </row>
@@ -1017,7 +997,7 @@
       <c r="A16">
         <v>2014</v>
       </c>
-      <c r="B16" s="2">
+      <c r="B16" s="1">
         <v>13617553</v>
       </c>
     </row>
@@ -1025,7 +1005,7 @@
       <c r="A17">
         <v>2015</v>
       </c>
-      <c r="B17" s="2">
+      <c r="B17" s="1">
         <v>13707118</v>
       </c>
     </row>
@@ -1033,7 +1013,7 @@
       <c r="A18">
         <v>2016</v>
       </c>
-      <c r="B18" s="2">
+      <c r="B18" s="1">
         <v>13875394</v>
       </c>
     </row>
@@ -1041,7 +1021,7 @@
       <c r="A19">
         <v>2017</v>
       </c>
-      <c r="B19" s="2">
+      <c r="B19" s="1">
         <v>14070141</v>
       </c>
     </row>
@@ -1049,7 +1029,7 @@
       <c r="A20">
         <v>2018</v>
       </c>
-      <c r="B20" s="2">
+      <c r="B20" s="1">
         <v>14308697</v>
       </c>
     </row>
@@ -1057,7 +1037,7 @@
       <c r="A21">
         <v>2019</v>
       </c>
-      <c r="B21" s="2">
+      <c r="B21" s="1">
         <v>14544701</v>
       </c>
     </row>
@@ -1065,7 +1045,7 @@
       <c r="A22">
         <v>2020</v>
       </c>
-      <c r="B22" s="2">
+      <c r="B22" s="1">
         <v>14726022</v>
       </c>
     </row>
@@ -1073,7 +1053,7 @@
       <c r="A23">
         <v>2021</v>
       </c>
-      <c r="B23" s="2">
+      <c r="B23" s="1">
         <v>14809257</v>
       </c>
     </row>
@@ -1081,7 +1061,7 @@
       <c r="A24">
         <v>2022</v>
       </c>
-      <c r="B24" s="2">
+      <c r="B24" s="1">
         <v>15109416</v>
       </c>
     </row>
@@ -1089,7 +1069,7 @@
       <c r="A25">
         <v>2023</v>
       </c>
-      <c r="B25" s="2">
+      <c r="B25" s="1">
         <v>15372100</v>
       </c>
     </row>
@@ -1097,7 +1077,7 @@
       <c r="A26">
         <v>2024</v>
       </c>
-      <c r="B26" s="2">
+      <c r="B26" s="1">
         <v>15610000</v>
       </c>
     </row>
@@ -1105,7 +1085,7 @@
       <c r="A27">
         <v>2025</v>
       </c>
-      <c r="B27" s="2">
+      <c r="B27" s="1">
         <v>15837800</v>
       </c>
     </row>
@@ -1113,7 +1093,7 @@
       <c r="A28">
         <v>2026</v>
       </c>
-      <c r="B28" s="2">
+      <c r="B28" s="1">
         <v>16058400</v>
       </c>
     </row>
@@ -1121,7 +1101,7 @@
       <c r="A29">
         <v>2027</v>
       </c>
-      <c r="B29" s="2">
+      <c r="B29" s="1">
         <v>16272600</v>
       </c>
     </row>
@@ -1129,23 +1109,23 @@
       <c r="A30">
         <v>2028</v>
       </c>
-      <c r="B30" s="2">
-        <v>16481400.000000002</v>
+      <c r="B30" s="1">
+        <v>16481400</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>2029</v>
       </c>
-      <c r="B31" s="2">
-        <v>16685099.999999998</v>
+      <c r="B31" s="1">
+        <v>16685100</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>2030</v>
       </c>
-      <c r="B32" s="2">
+      <c r="B32" s="1">
         <v>16883800</v>
       </c>
     </row>
@@ -1153,7 +1133,7 @@
       <c r="A33">
         <v>2031</v>
       </c>
-      <c r="B33" s="2">
+      <c r="B33" s="1">
         <v>17077600</v>
       </c>
     </row>
@@ -1161,7 +1141,7 @@
       <c r="A34">
         <v>2032</v>
       </c>
-      <c r="B34" s="2">
+      <c r="B34" s="1">
         <v>17267200</v>
       </c>
     </row>
@@ -1169,7 +1149,7 @@
       <c r="A35">
         <v>2033</v>
       </c>
-      <c r="B35" s="2">
+      <c r="B35" s="1">
         <v>17452100</v>
       </c>
     </row>
@@ -1177,7 +1157,7 @@
       <c r="A36">
         <v>2034</v>
       </c>
-      <c r="B36" s="2">
+      <c r="B36" s="1">
         <v>17632000</v>
       </c>
     </row>
@@ -1185,7 +1165,7 @@
       <c r="A37">
         <v>2035</v>
       </c>
-      <c r="B37" s="2">
+      <c r="B37" s="1">
         <v>17807200</v>
       </c>
     </row>
@@ -1193,7 +1173,7 @@
       <c r="A38">
         <v>2036</v>
       </c>
-      <c r="B38" s="2">
+      <c r="B38" s="1">
         <v>17977400</v>
       </c>
     </row>
@@ -1201,7 +1181,7 @@
       <c r="A39">
         <v>2037</v>
       </c>
-      <c r="B39" s="2">
+      <c r="B39" s="1">
         <v>18143000</v>
       </c>
     </row>
@@ -1209,7 +1189,7 @@
       <c r="A40">
         <v>2038</v>
       </c>
-      <c r="B40" s="2">
+      <c r="B40" s="1">
         <v>18304200</v>
       </c>
     </row>
@@ -1217,7 +1197,7 @@
       <c r="A41">
         <v>2039</v>
       </c>
-      <c r="B41" s="2">
+      <c r="B41" s="1">
         <v>18461400</v>
       </c>
     </row>
@@ -1225,7 +1205,7 @@
       <c r="A42">
         <v>2040</v>
       </c>
-      <c r="B42" s="2">
+      <c r="B42" s="1">
         <v>18615400</v>
       </c>
     </row>
@@ -1233,7 +1213,7 @@
       <c r="A43">
         <v>2041</v>
       </c>
-      <c r="B43" s="2">
+      <c r="B43" s="1">
         <v>18766700</v>
       </c>
     </row>
@@ -1241,7 +1221,7 @@
       <c r="A44">
         <v>2042</v>
       </c>
-      <c r="B44" s="2">
+      <c r="B44" s="1">
         <v>18916400</v>
       </c>
     </row>
@@ -1249,7 +1229,7 @@
       <c r="A45">
         <v>2043</v>
       </c>
-      <c r="B45" s="2">
+      <c r="B45" s="1">
         <v>19065300</v>
       </c>
     </row>
@@ -1257,7 +1237,7 @@
       <c r="A46">
         <v>2044</v>
       </c>
-      <c r="B46" s="2">
+      <c r="B46" s="1">
         <v>19201200</v>
       </c>
     </row>
@@ -1265,7 +1245,7 @@
       <c r="A47">
         <v>2045</v>
       </c>
-      <c r="B47" s="2">
+      <c r="B47" s="1">
         <v>19336000</v>
       </c>
     </row>
@@ -1273,7 +1253,7 @@
       <c r="A48">
         <v>2046</v>
       </c>
-      <c r="B48" s="2">
+      <c r="B48" s="1">
         <v>19469800</v>
       </c>
     </row>
@@ -1281,7 +1261,7 @@
       <c r="A49">
         <v>2047</v>
       </c>
-      <c r="B49" s="2">
+      <c r="B49" s="1">
         <v>19602700</v>
       </c>
     </row>
@@ -1289,7 +1269,7 @@
       <c r="A50">
         <v>2048</v>
       </c>
-      <c r="B50" s="2">
+      <c r="B50" s="1">
         <v>19734700</v>
       </c>
     </row>
@@ -1297,7 +1277,7 @@
       <c r="A51">
         <v>2049</v>
       </c>
-      <c r="B51" s="2">
+      <c r="B51" s="1">
         <v>19866100</v>
       </c>
     </row>
@@ -1305,12 +1285,11 @@
       <c r="A52">
         <v>2050</v>
       </c>
-      <c r="B52" s="2">
+      <c r="B52" s="1">
         <v>19997000</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
finished lighting subsector... such as it is
</commit_message>
<xml_diff>
--- a/input_files/population.xlsx
+++ b/input_files/population.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://utoronto-my.sharepoint.com/personal/ian_elder_mail_utoronto_ca/Documents/Documents/TEMOA/buildings_sector/input_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{A1F4FCB6-EB9F-435E-A7B8-638927D142CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9D9EDC5-462A-4425-8F34-5DB64C00047F}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{A1F4FCB6-EB9F-435E-A7B8-638927D142CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F2810BE-236B-474C-A9BC-A82ACEF9C0F0}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="on" sheetId="1" r:id="rId1"/>
+    <sheet name="ON" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>

</xml_diff>

<commit_message>
Got model running. Added population index aggregation, tested BC (working)
</commit_message>
<xml_diff>
--- a/input_files/population.xlsx
+++ b/input_files/population.xlsx
@@ -8,15 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://utoronto-my.sharepoint.com/personal/ian_elder_mail_utoronto_ca/Documents/Documents/TEMOA/buildings_sector/input_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{A1F4FCB6-EB9F-435E-A7B8-638927D142CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{615BAB8F-82F4-469E-A3B3-02F613258B34}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{A1F4FCB6-EB9F-435E-A7B8-638927D142CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{648D3CCB-E69F-40E6-B95A-04C4AE1B686B}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-13740" yWindow="3585" windowWidth="21600" windowHeight="11385" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ON" sheetId="1" r:id="rId1"/>
     <sheet name="AB" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 

</xml_diff>